<commit_message>
fix xlsx load in mapper editor
</commit_message>
<xml_diff>
--- a/data/ab-2.xlsx
+++ b/data/ab-2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dane\Projects\Quickport\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7C36F20-CA40-4ADB-BA35-A2FBF6746BB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FD6354B-C422-4D9E-9C3A-B26A17689A0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{28EB59AA-5D23-0345-8BB0-371A52075FE6}"/>
   </bookViews>
@@ -370,7 +370,47 @@
     <cellStyle name="Procentowy" xfId="2" builtinId="5"/>
     <cellStyle name="Walutowy" xfId="1" builtinId="4"/>
   </cellStyles>
-  <dxfs count="34">
+  <dxfs count="38">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -656,44 +696,44 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1E398AED-A032-5141-BD97-02F58A0B9452}" name="Table13" displayName="Table13" ref="B3:N6" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1E398AED-A032-5141-BD97-02F58A0B9452}" name="Table13" displayName="Table13" ref="B3:N6" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
   <autoFilter ref="B3:N6" xr:uid="{1E398AED-A032-5141-BD97-02F58A0B9452}"/>
   <tableColumns count="13">
-    <tableColumn id="15" xr3:uid="{82C2CD33-72ED-834D-8D91-B3AB103B80B5}" name="Update Status" dataDxfId="31"/>
-    <tableColumn id="16" xr3:uid="{CDD66C4F-187A-5B41-AB33-3633BD033394}" name="Effective Date" dataDxfId="30"/>
+    <tableColumn id="15" xr3:uid="{82C2CD33-72ED-834D-8D91-B3AB103B80B5}" name="Update Status" dataDxfId="35"/>
+    <tableColumn id="16" xr3:uid="{CDD66C4F-187A-5B41-AB33-3633BD033394}" name="Effective Date" dataDxfId="34"/>
     <tableColumn id="1" xr3:uid="{6ABB9F36-AB5C-CB48-B65E-ACD803F71C9F}" name="Name"/>
-    <tableColumn id="2" xr3:uid="{748E55DF-3109-464E-A93D-D84763BB4F74}" name="Restricted" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{F7D38490-1DC4-0644-9093-0AC15C001515}" name="Category" dataDxfId="28"/>
-    <tableColumn id="4" xr3:uid="{AD68A147-7A7D-2749-BA72-A54189B73218}" name="UPC" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{E246E2E5-6DC9-044D-B53F-925AE6A3486D}" name="SKU" dataDxfId="26"/>
-    <tableColumn id="6" xr3:uid="{A0C53757-7DFD-9640-8E85-71A84BAFB2DD}" name="MSRP" dataDxfId="25"/>
-    <tableColumn id="7" xr3:uid="{FF99DF05-2AD0-F846-9889-B4FDE410EC3E}" name="Method of Delivery" dataDxfId="24"/>
-    <tableColumn id="8" xr3:uid="{5B98F000-A041-8A48-A75B-6203FB7C7206}" name="Dimensions of _x000a_unit in box_x000a_(inches)" dataDxfId="23"/>
-    <tableColumn id="9" xr3:uid="{2CE3789B-13A7-6144-AEA6-32C3236BA9B7}" name="Weight of _x000a_unit in box (LBS)" dataDxfId="22"/>
-    <tableColumn id="10" xr3:uid="{6EF3F2E8-F654-C449-82E1-10989C25A5CD}" name="Product Family" dataDxfId="21"/>
-    <tableColumn id="11" xr3:uid="{E24FD614-FCD1-3E4A-AC8E-A22167A484A3}" name="Product Group" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{748E55DF-3109-464E-A93D-D84763BB4F74}" name="Restricted" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{F7D38490-1DC4-0644-9093-0AC15C001515}" name="Category" dataDxfId="32"/>
+    <tableColumn id="4" xr3:uid="{AD68A147-7A7D-2749-BA72-A54189B73218}" name="UPC" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{E246E2E5-6DC9-044D-B53F-925AE6A3486D}" name="SKU" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{A0C53757-7DFD-9640-8E85-71A84BAFB2DD}" name="MSRP" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{FF99DF05-2AD0-F846-9889-B4FDE410EC3E}" name="Method of Delivery" dataDxfId="28"/>
+    <tableColumn id="8" xr3:uid="{5B98F000-A041-8A48-A75B-6203FB7C7206}" name="Dimensions of _x000a_unit in box_x000a_(inches)" dataDxfId="27"/>
+    <tableColumn id="9" xr3:uid="{2CE3789B-13A7-6144-AEA6-32C3236BA9B7}" name="Weight of _x000a_unit in box (LBS)" dataDxfId="26"/>
+    <tableColumn id="10" xr3:uid="{6EF3F2E8-F654-C449-82E1-10989C25A5CD}" name="Product Family" dataDxfId="25"/>
+    <tableColumn id="11" xr3:uid="{E24FD614-FCD1-3E4A-AC8E-A22167A484A3}" name="Product Group" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1AA81F91-0962-9641-89E5-FD3D02220D37}" name="Table1" displayName="Table1" ref="B3:N10" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1AA81F91-0962-9641-89E5-FD3D02220D37}" name="Table1" displayName="Table1" ref="B3:N10" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
   <autoFilter ref="B3:N10" xr:uid="{1AA81F91-0962-9641-89E5-FD3D02220D37}"/>
   <tableColumns count="13">
-    <tableColumn id="15" xr3:uid="{B0EE1426-39B0-444F-B073-17B7C409C02A}" name="Update Status" dataDxfId="17"/>
-    <tableColumn id="16" xr3:uid="{58DDAA30-B9C2-6C4C-A412-B4C89D4A45BC}" name="Effective Date" dataDxfId="16"/>
-    <tableColumn id="1" xr3:uid="{B4ABDCCB-59DD-E345-AB1A-6128E1E41249}" name="Name" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{8A8EB213-0E18-5541-B9BE-CA9C85E7377C}" name="Restricted" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{A5081C7E-E8BB-AF42-A998-FFF5A18BAB6D}" name="Category" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{2C5A191E-8FF0-4848-9E51-5F9F3E5DE2AF}" name="UPC" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{043401D6-231C-0248-98A0-991A5237A79A}" name="SKU" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{F79EE368-9474-F34D-8F3A-3310290B247E}" name="MSRP" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{02AC31D4-9368-6542-9C78-F5733864632C}" name="Method of Delivery" dataDxfId="9"/>
-    <tableColumn id="8" xr3:uid="{B94C8957-4325-0844-9230-44F565E71653}" name="Dimensions of _x000a_unit in box_x000a_(inches)" dataDxfId="8"/>
-    <tableColumn id="9" xr3:uid="{8A5E7461-0EB9-8145-A5B5-BFAAD4347438}" name="Weight of _x000a_unit in box (LBS)" dataDxfId="7"/>
-    <tableColumn id="10" xr3:uid="{7E93A410-C614-FA47-9EF2-D7753F5A10CA}" name="Product Family" dataDxfId="6"/>
-    <tableColumn id="11" xr3:uid="{50171BDB-2839-E646-9EFD-B1D9A9D90B26}" name="Product Group" dataDxfId="5"/>
+    <tableColumn id="15" xr3:uid="{B0EE1426-39B0-444F-B073-17B7C409C02A}" name="Update Status" dataDxfId="21"/>
+    <tableColumn id="16" xr3:uid="{58DDAA30-B9C2-6C4C-A412-B4C89D4A45BC}" name="Effective Date" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{B4ABDCCB-59DD-E345-AB1A-6128E1E41249}" name="Name" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{8A8EB213-0E18-5541-B9BE-CA9C85E7377C}" name="Restricted" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{A5081C7E-E8BB-AF42-A998-FFF5A18BAB6D}" name="Category" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{2C5A191E-8FF0-4848-9E51-5F9F3E5DE2AF}" name="UPC" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{043401D6-231C-0248-98A0-991A5237A79A}" name="SKU" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{F79EE368-9474-F34D-8F3A-3310290B247E}" name="MSRP" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{02AC31D4-9368-6542-9C78-F5733864632C}" name="Method of Delivery" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{B94C8957-4325-0844-9230-44F565E71653}" name="Dimensions of _x000a_unit in box_x000a_(inches)" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{8A5E7461-0EB9-8145-A5B5-BFAAD4347438}" name="Weight of _x000a_unit in box (LBS)" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{7E93A410-C614-FA47-9EF2-D7753F5A10CA}" name="Product Family" dataDxfId="10"/>
+    <tableColumn id="11" xr3:uid="{50171BDB-2839-E646-9EFD-B1D9A9D90B26}" name="Product Group" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2752,8 +2792,8 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="H4:H6">
-    <cfRule type="duplicateValues" dxfId="4" priority="20"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="21"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -3026,9 +3066,9 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="H4:H10">
-    <cfRule type="duplicateValues" dxfId="2" priority="17"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="18"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="19"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
renamed views to presenters, fixed icons and images
</commit_message>
<xml_diff>
--- a/data/ab-2.xlsx
+++ b/data/ab-2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dane\Projects\Quickport\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FD6354B-C422-4D9E-9C3A-B26A17689A0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC24EF9D-5E14-4AAF-A81F-65FF06F3F588}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{28EB59AA-5D23-0345-8BB0-371A52075FE6}"/>
+    <workbookView xWindow="5895" yWindow="4440" windowWidth="22905" windowHeight="11040" xr2:uid="{28EB59AA-5D23-0345-8BB0-371A52075FE6}"/>
   </bookViews>
   <sheets>
     <sheet name="renewals" sheetId="1" r:id="rId1"/>
@@ -365,10 +365,10 @@
     </xf>
   </cellXfs>
   <cellStyles count="4">
-    <cellStyle name="Currency" xfId="1" builtinId="4"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal_eSeries Price list" xfId="3" xr:uid="{37CAD8B9-A931-254A-8FF3-78E05189BE48}"/>
-    <cellStyle name="Percent" xfId="2" builtinId="5"/>
+    <cellStyle name="Normalny" xfId="0" builtinId="0"/>
+    <cellStyle name="Procentowy" xfId="2" builtinId="5"/>
+    <cellStyle name="Walutowy" xfId="1" builtinId="4"/>
   </cellStyles>
   <dxfs count="34">
     <dxf>
@@ -700,9 +700,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Motyw pakietu Office">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Pakiet Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -740,7 +740,7 @@
         <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Pakiet Office">
       <a:majorFont>
         <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
@@ -846,7 +846,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Pakiet Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1017,21 +1017,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E648E21-2D13-3347-8F10-8AE3CE884464}">
   <dimension ref="B1:N1537"/>
-  <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="15.6"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="3.5" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.3984375" style="20" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.375" style="20" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="97.5" style="20" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15" style="20" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.59765625" style="20" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.625" style="20" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.5" style="22" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.5" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="12.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="16.5" style="5" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="18" style="5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.59765625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.59765625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:14" s="7" customFormat="1">
@@ -1062,7 +1062,7 @@
       <c r="K2" s="8"/>
       <c r="L2" s="8"/>
     </row>
-    <row r="3" spans="2:14" ht="43.2">
+    <row r="3" spans="2:14" ht="45">
       <c r="B3" s="9" t="s">
         <v>0</v>
       </c>
@@ -1118,7 +1118,7 @@
         <v>32</v>
       </c>
       <c r="I4" s="18">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>14</v>
@@ -2765,21 +2765,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B45CD3DC-862A-EF46-9C41-67353FA0D813}">
   <dimension ref="B1:N10"/>
-  <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="15.6"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="3.5" customWidth="1"/>
-    <col min="2" max="2" width="25.09765625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.3984375" style="20" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.375" style="20" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="82.5" style="20" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15" style="20" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.59765625" style="20" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.625" style="20" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.5" style="22" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.5" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.3984375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="15.375" style="5" customWidth="1"/>
     <col min="12" max="12" width="12.5" style="5" customWidth="1"/>
-    <col min="13" max="13" width="16.3984375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="26.09765625" customWidth="1"/>
+    <col min="13" max="13" width="16.375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="26.125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:14" s="7" customFormat="1">
@@ -2810,7 +2810,7 @@
       <c r="K2" s="8"/>
       <c r="L2" s="8"/>
     </row>
-    <row r="3" spans="2:14" ht="43.2">
+    <row r="3" spans="2:14" ht="45">
       <c r="B3" s="9" t="s">
         <v>0</v>
       </c>

</xml_diff>